<commit_message>
chore(pricing): agreement.csv + reconciled outputs (engines wired: 51/63 cuts agreed, 12 held)
Engine wiring live: pricing engine emits agreement.csv; tracker holds the 12
waste-cuts the cross-price optimizer disagrees with (9 hold, 3 raise), cutting
only the 51 both-engines-agree. Run-stamped history/ kept local (gitignored).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
+++ b/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
@@ -6681,50 +6681,50 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="9" t="inlineStr">
+      <c r="A133" s="4" t="inlineStr">
         <is>
           <t>Flax Seeds</t>
         </is>
       </c>
-      <c r="B133" s="10" t="inlineStr">
+      <c r="B133" s="5" t="inlineStr">
         <is>
           <t>Lucknow</t>
         </is>
       </c>
-      <c r="C133" s="9" t="inlineStr">
+      <c r="C133" s="4" t="inlineStr">
         <is>
           <t>Seeds</t>
         </is>
       </c>
-      <c r="D133" s="11" t="n">
+      <c r="D133" s="6" t="n">
         <v>78.8</v>
       </c>
-      <c r="E133" s="12" t="n">
+      <c r="E133" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="F133" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G133" s="11" t="n">
-        <v>80</v>
-      </c>
-      <c r="H133" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I133" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J133" s="13" t="inlineStr">
-        <is>
-          <t>discount 2% reliably below break-even — even the optimistic CI of its effect (marg β -0.0314 vs pay-threshold 0.0101) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K133" s="11" t="n">
-        <v>7.439999999999998</v>
+      <c r="F133" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G133" s="6" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I133" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J133" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K133" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -11146,50 +11146,50 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="9" t="inlineStr">
+      <c r="A228" s="4" t="inlineStr">
         <is>
           <t>Jaggery Powder 500 g</t>
         </is>
       </c>
-      <c r="B228" s="10" t="inlineStr">
+      <c r="B228" s="5" t="inlineStr">
         <is>
           <t>Chandigarh Tricity</t>
         </is>
       </c>
-      <c r="C228" s="9" t="inlineStr">
+      <c r="C228" s="4" t="inlineStr">
         <is>
           <t>Jaggery</t>
         </is>
       </c>
-      <c r="D228" s="11" t="n">
+      <c r="D228" s="6" t="n">
         <v>82.44</v>
       </c>
-      <c r="E228" s="12" t="n">
+      <c r="E228" s="7" t="n">
         <v>8.4</v>
       </c>
-      <c r="F228" s="12" t="n">
-        <v>7.12</v>
-      </c>
-      <c r="G228" s="11" t="n">
-        <v>83.592</v>
-      </c>
-      <c r="H228" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I228" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J228" s="13" t="inlineStr">
-        <is>
-          <t>discount 8% reliably below break-even — even the optimistic CI of its effect (marg β -0.0084 vs pay-threshold 0.0109) doesn't pay; trim to 7% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K228" s="11" t="n">
-        <v>140.7744000000002</v>
+      <c r="F228" s="7" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G228" s="6" t="n">
+        <v>82.44</v>
+      </c>
+      <c r="H228" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I228" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J228" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K228" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="229">
@@ -11334,50 +11334,50 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="9" t="inlineStr">
+      <c r="A232" s="4" t="inlineStr">
         <is>
           <t>Jaggery Powder 500 g</t>
         </is>
       </c>
-      <c r="B232" s="10" t="inlineStr">
+      <c r="B232" s="5" t="inlineStr">
         <is>
           <t>Kolkata</t>
         </is>
       </c>
-      <c r="C232" s="9" t="inlineStr">
+      <c r="C232" s="4" t="inlineStr">
         <is>
           <t>Jaggery</t>
         </is>
       </c>
-      <c r="D232" s="11" t="n">
+      <c r="D232" s="6" t="n">
         <v>82.14</v>
       </c>
-      <c r="E232" s="12" t="n">
+      <c r="E232" s="7" t="n">
         <v>8.73</v>
       </c>
-      <c r="F232" s="12" t="n">
-        <v>7.12</v>
-      </c>
-      <c r="G232" s="11" t="n">
-        <v>83.592</v>
-      </c>
-      <c r="H232" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I232" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J232" s="13" t="inlineStr">
-        <is>
-          <t>discount 9% reliably below break-even — even the optimistic CI of its effect (marg β -0.0081 vs pay-threshold 0.0110) doesn't pay; trim to 7% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K232" s="11" t="n">
-        <v>1129.946400000001</v>
+      <c r="F232" s="7" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="G232" s="6" t="n">
+        <v>82.143</v>
+      </c>
+      <c r="H232" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I232" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J232" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K232" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="233">
@@ -18478,50 +18478,50 @@
       </c>
     </row>
     <row r="384">
-      <c r="A384" s="9" t="inlineStr">
+      <c r="A384" s="4" t="inlineStr">
         <is>
           <t>Low GI Rice</t>
         </is>
       </c>
-      <c r="B384" s="10" t="inlineStr">
+      <c r="B384" s="5" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="C384" s="9" t="inlineStr">
+      <c r="C384" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D384" s="11" t="n">
+      <c r="D384" s="6" t="n">
         <v>573.77</v>
       </c>
-      <c r="E384" s="12" t="n">
+      <c r="E384" s="7" t="n">
         <v>23.5</v>
       </c>
-      <c r="F384" s="12" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="G384" s="11" t="n">
-        <v>596.25</v>
-      </c>
-      <c r="H384" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I384" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J384" s="13" t="inlineStr">
-        <is>
-          <t>discount 24% reliably below break-even — even the optimistic CI of its effect (marg β -0.0046 vs pay-threshold 0.0131) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K384" s="11" t="n">
-        <v>1227.357482698962</v>
+      <c r="F384" s="7" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="G384" s="6" t="n">
+        <v>573.75</v>
+      </c>
+      <c r="H384" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I384" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J384" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K384" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="385">
@@ -18666,50 +18666,50 @@
       </c>
     </row>
     <row r="388">
-      <c r="A388" s="9" t="inlineStr">
+      <c r="A388" s="4" t="inlineStr">
         <is>
           <t>Low GI Rice</t>
         </is>
       </c>
-      <c r="B388" s="10" t="inlineStr">
+      <c r="B388" s="5" t="inlineStr">
         <is>
           <t>Kolkata</t>
         </is>
       </c>
-      <c r="C388" s="9" t="inlineStr">
+      <c r="C388" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D388" s="11" t="n">
+      <c r="D388" s="6" t="n">
         <v>583.4</v>
       </c>
-      <c r="E388" s="12" t="n">
+      <c r="E388" s="7" t="n">
         <v>22.21</v>
       </c>
-      <c r="F388" s="12" t="n">
-        <v>19.21</v>
-      </c>
-      <c r="G388" s="11" t="n">
-        <v>605.925</v>
-      </c>
-      <c r="H388" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I388" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J388" s="13" t="inlineStr">
-        <is>
-          <t>discount 22% reliably below break-even — even the optimistic CI of its effect (marg β -0.0038 vs pay-threshold 0.0129) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K388" s="11" t="n">
-        <v>505.0519926706364</v>
+      <c r="F388" s="7" t="n">
+        <v>22.21</v>
+      </c>
+      <c r="G388" s="6" t="n">
+        <v>583.4250000000001</v>
+      </c>
+      <c r="H388" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I388" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J388" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K388" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="389">
@@ -22332,50 +22332,50 @@
       </c>
     </row>
     <row r="466">
-      <c r="A466" s="9" t="inlineStr">
+      <c r="A466" s="4" t="inlineStr">
         <is>
           <t>Active Mantras Organic Low GI Rice</t>
         </is>
       </c>
-      <c r="B466" s="10" t="inlineStr">
+      <c r="B466" s="5" t="inlineStr">
         <is>
           <t>Lucknow</t>
         </is>
       </c>
-      <c r="C466" s="9" t="inlineStr">
+      <c r="C466" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D466" s="11" t="n">
+      <c r="D466" s="6" t="n">
         <v>130.08</v>
       </c>
-      <c r="E466" s="12" t="n">
+      <c r="E466" s="7" t="n">
         <v>13.28</v>
       </c>
-      <c r="F466" s="12" t="n">
-        <v>10.28</v>
-      </c>
-      <c r="G466" s="11" t="n">
-        <v>134.58</v>
-      </c>
-      <c r="H466" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I466" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J466" s="13" t="inlineStr">
-        <is>
-          <t>discount 13% reliably below break-even — even the optimistic CI of its effect (marg β +0.0015 vs pay-threshold 0.0115) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K466" s="11" t="n">
-        <v>14.12441860465117</v>
+      <c r="F466" s="7" t="n">
+        <v>13.28</v>
+      </c>
+      <c r="G466" s="6" t="n">
+        <v>130.08</v>
+      </c>
+      <c r="H466" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I466" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J466" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K466" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="467">
@@ -23554,50 +23554,50 @@
       </c>
     </row>
     <row r="492">
-      <c r="A492" s="9" t="inlineStr">
+      <c r="A492" s="4" t="inlineStr">
         <is>
           <t>Brown Sonamasuri Rice</t>
         </is>
       </c>
-      <c r="B492" s="10" t="inlineStr">
+      <c r="B492" s="5" t="inlineStr">
         <is>
           <t>Chandigarh Tricity</t>
         </is>
       </c>
-      <c r="C492" s="9" t="inlineStr">
+      <c r="C492" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D492" s="11" t="n">
+      <c r="D492" s="6" t="n">
         <v>110.59</v>
       </c>
-      <c r="E492" s="12" t="n">
+      <c r="E492" s="7" t="n">
         <v>14.93</v>
       </c>
-      <c r="F492" s="12" t="n">
-        <v>11.93</v>
-      </c>
-      <c r="G492" s="11" t="n">
-        <v>114.491</v>
-      </c>
-      <c r="H492" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I492" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J492" s="13" t="inlineStr">
-        <is>
-          <t>discount 15% reliably below break-even — even the optimistic CI of its effect (marg β +0.0006 vs pay-threshold 0.0118) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K492" s="11" t="n">
-        <v>34.71072164948453</v>
+      <c r="F492" s="7" t="n">
+        <v>14.93</v>
+      </c>
+      <c r="G492" s="6" t="n">
+        <v>110.591</v>
+      </c>
+      <c r="H492" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I492" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J492" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K492" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="493">
@@ -23883,50 +23883,50 @@
       </c>
     </row>
     <row r="499">
-      <c r="A499" s="9" t="inlineStr">
+      <c r="A499" s="4" t="inlineStr">
         <is>
           <t>Brown Sonamasuri Rice</t>
         </is>
       </c>
-      <c r="B499" s="10" t="inlineStr">
+      <c r="B499" s="5" t="inlineStr">
         <is>
           <t>Others</t>
         </is>
       </c>
-      <c r="C499" s="9" t="inlineStr">
+      <c r="C499" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D499" s="11" t="n">
+      <c r="D499" s="6" t="n">
         <v>110.66</v>
       </c>
-      <c r="E499" s="12" t="n">
+      <c r="E499" s="7" t="n">
         <v>14.88</v>
       </c>
-      <c r="F499" s="12" t="n">
-        <v>11.88</v>
-      </c>
-      <c r="G499" s="11" t="n">
-        <v>114.556</v>
-      </c>
-      <c r="H499" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I499" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J499" s="13" t="inlineStr">
-        <is>
-          <t>discount 15% reliably below break-even — even the optimistic CI of its effect (marg β +0.0006 vs pay-threshold 0.0118) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K499" s="11" t="n">
-        <v>1165.851310344828</v>
+      <c r="F499" s="7" t="n">
+        <v>14.88</v>
+      </c>
+      <c r="G499" s="6" t="n">
+        <v>110.656</v>
+      </c>
+      <c r="H499" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I499" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J499" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K499" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="500">
@@ -25857,50 +25857,50 @@
       </c>
     </row>
     <row r="541">
-      <c r="A541" s="9" t="inlineStr">
+      <c r="A541" s="4" t="inlineStr">
         <is>
           <t>Sonamasuri Rice</t>
         </is>
       </c>
-      <c r="B541" s="10" t="inlineStr">
+      <c r="B541" s="5" t="inlineStr">
         <is>
           <t>Chandigarh Tricity</t>
         </is>
       </c>
-      <c r="C541" s="9" t="inlineStr">
+      <c r="C541" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D541" s="11" t="n">
+      <c r="D541" s="6" t="n">
         <v>491.33</v>
       </c>
-      <c r="E541" s="12" t="n">
+      <c r="E541" s="7" t="n">
         <v>17.98</v>
       </c>
-      <c r="F541" s="12" t="n">
-        <v>14.98</v>
-      </c>
-      <c r="G541" s="11" t="n">
-        <v>509.2698</v>
-      </c>
-      <c r="H541" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I541" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J541" s="13" t="inlineStr">
-        <is>
-          <t>discount 18% reliably below break-even — even the optimistic CI of its effect (marg β -0.0013 vs pay-threshold 0.0122) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K541" s="11" t="n">
-        <v>108.4485238636364</v>
+      <c r="F541" s="7" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="G541" s="6" t="n">
+        <v>491.2998</v>
+      </c>
+      <c r="H541" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I541" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J541" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K541" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="542">
@@ -25951,50 +25951,50 @@
       </c>
     </row>
     <row r="543">
-      <c r="A543" s="9" t="inlineStr">
+      <c r="A543" s="4" t="inlineStr">
         <is>
           <t>Sonamasuri Rice</t>
         </is>
       </c>
-      <c r="B543" s="10" t="inlineStr">
+      <c r="B543" s="5" t="inlineStr">
         <is>
           <t>Delhi-NCR</t>
         </is>
       </c>
-      <c r="C543" s="9" t="inlineStr">
+      <c r="C543" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D543" s="11" t="n">
+      <c r="D543" s="6" t="n">
         <v>493.7</v>
       </c>
-      <c r="E543" s="12" t="n">
+      <c r="E543" s="7" t="n">
         <v>17.58</v>
       </c>
-      <c r="F543" s="12" t="n">
-        <v>14.58</v>
-      </c>
-      <c r="G543" s="11" t="n">
-        <v>511.6658</v>
-      </c>
-      <c r="H543" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I543" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J543" s="13" t="inlineStr">
-        <is>
-          <t>discount 18% reliably below break-even — even the optimistic CI of its effect (marg β -0.0010 vs pay-threshold 0.0121) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K543" s="11" t="n">
-        <v>1390.60511860465</v>
+      <c r="F543" s="7" t="n">
+        <v>17.58</v>
+      </c>
+      <c r="G543" s="6" t="n">
+        <v>493.6958</v>
+      </c>
+      <c r="H543" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I543" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J543" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K543" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="544">
@@ -26045,50 +26045,50 @@
       </c>
     </row>
     <row r="545">
-      <c r="A545" s="9" t="inlineStr">
+      <c r="A545" s="4" t="inlineStr">
         <is>
           <t>Sonamasuri Rice</t>
         </is>
       </c>
-      <c r="B545" s="10" t="inlineStr">
+      <c r="B545" s="5" t="inlineStr">
         <is>
           <t>Kolkata</t>
         </is>
       </c>
-      <c r="C545" s="9" t="inlineStr">
+      <c r="C545" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D545" s="11" t="n">
+      <c r="D545" s="6" t="n">
         <v>494.75</v>
       </c>
-      <c r="E545" s="12" t="n">
+      <c r="E545" s="7" t="n">
         <v>17.4</v>
       </c>
-      <c r="F545" s="12" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="G545" s="11" t="n">
-        <v>512.744</v>
-      </c>
-      <c r="H545" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I545" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J545" s="13" t="inlineStr">
-        <is>
-          <t>discount 17% reliably below break-even — even the optimistic CI of its effect (marg β -0.0009 vs pay-threshold 0.0121) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K545" s="11" t="n">
-        <v>479.1860975323152</v>
+      <c r="F545" s="7" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="G545" s="6" t="n">
+        <v>494.7740000000001</v>
+      </c>
+      <c r="H545" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I545" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J545" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K545" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="546">
@@ -26233,50 +26233,50 @@
       </c>
     </row>
     <row r="549">
-      <c r="A549" s="9" t="inlineStr">
+      <c r="A549" s="4" t="inlineStr">
         <is>
           <t>Sonamasuri Rice</t>
         </is>
       </c>
-      <c r="B549" s="10" t="inlineStr">
+      <c r="B549" s="5" t="inlineStr">
         <is>
           <t>Pune</t>
         </is>
       </c>
-      <c r="C549" s="9" t="inlineStr">
+      <c r="C549" s="4" t="inlineStr">
         <is>
           <t>Rice &amp; Rice Products</t>
         </is>
       </c>
-      <c r="D549" s="11" t="n">
+      <c r="D549" s="6" t="n">
         <v>492.98</v>
       </c>
-      <c r="E549" s="12" t="n">
+      <c r="E549" s="7" t="n">
         <v>17.7</v>
       </c>
-      <c r="F549" s="12" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="G549" s="11" t="n">
-        <v>510.947</v>
-      </c>
-      <c r="H549" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I549" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J549" s="13" t="inlineStr">
-        <is>
-          <t>discount 18% reliably below break-even — even the optimistic CI of its effect (marg β -0.0011 vs pay-threshold 0.0121) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K549" s="11" t="n">
-        <v>228.617289838337</v>
+      <c r="F549" s="7" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G549" s="6" t="n">
+        <v>492.977</v>
+      </c>
+      <c r="H549" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I549" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J549" s="8" t="inlineStr">
+        <is>
+          <t>engines disagree - test first</t>
+        </is>
+      </c>
+      <c r="K549" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="550">
@@ -28166,7 +28166,7 @@
         </is>
       </c>
       <c r="K590" s="15" t="n">
-        <v>39342.28346189268</v>
+        <v>32910.16970608517</v>
       </c>
     </row>
   </sheetData>
@@ -28224,7 +28224,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>1203934.3663</v>
+        <v>1213421.6965</v>
       </c>
     </row>
     <row r="6">
@@ -28234,7 +28234,7 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>13.44432991660488</v>
+        <v>13.55027489235016</v>
       </c>
     </row>
     <row r="7">
@@ -28254,7 +28254,7 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>50655.52970000007</v>
+        <v>41168.19949999987</v>
       </c>
     </row>
     <row r="9"/>

</xml_diff>

<commit_message>
feat(tracker): competitive-defense hold — keep challenger-flagged defense cells out of the cut wave
The champion/challenger pass reclassifies cells from c_waste_cut to competitive
defense (bucket c under Model A, not-c under Model B) where our discount was
holding the line against a rival promo, not pure waste. We KEEP champion Model A,
so these still read as waste-cut in the tracker; apply_defense_hold now reads
DISCOUNT_PLAN/defense_hold.csv and holds them out of the first cut wave (watch,
do not slash). challenger.py regenerates defense_hold.csv every retrain, so an
empty defense set correctly releases prior holds. Day-one state: cut 48 / hold
537 (3 defense cells + 12 engine-disagreement held), 585 W1 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
+++ b/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
@@ -7668,50 +7668,50 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="9" t="inlineStr">
+      <c r="A154" s="4" t="inlineStr">
         <is>
           <t>Chana Dal</t>
         </is>
       </c>
-      <c r="B154" s="10" t="inlineStr">
+      <c r="B154" s="5" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="C154" s="9" t="inlineStr">
+      <c r="C154" s="4" t="inlineStr">
         <is>
           <t>Dal &amp; Pulses</t>
         </is>
       </c>
-      <c r="D154" s="11" t="n">
+      <c r="D154" s="6" t="n">
         <v>103.01</v>
       </c>
-      <c r="E154" s="12" t="n">
+      <c r="E154" s="7" t="n">
         <v>16.25</v>
       </c>
-      <c r="F154" s="12" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="G154" s="11" t="n">
-        <v>106.7025</v>
-      </c>
-      <c r="H154" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I154" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J154" s="13" t="inlineStr">
-        <is>
-          <t>discount 16% reliably below break-even — even the optimistic CI of its effect (marg β +0.0030 vs pay-threshold 0.0119) doesn't pay; trim to 2% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K154" s="11" t="n">
-        <v>132.4529456521741</v>
+      <c r="F154" s="7" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="G154" s="6" t="n">
+        <v>103.0125</v>
+      </c>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I154" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J154" s="8" t="inlineStr">
+        <is>
+          <t>competitive defense - hold, do not cut</t>
+        </is>
+      </c>
+      <c r="K154" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="155">
@@ -7762,50 +7762,50 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="9" t="inlineStr">
+      <c r="A156" s="4" t="inlineStr">
         <is>
           <t>Chana Dal</t>
         </is>
       </c>
-      <c r="B156" s="10" t="inlineStr">
+      <c r="B156" s="5" t="inlineStr">
         <is>
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="C156" s="9" t="inlineStr">
+      <c r="C156" s="4" t="inlineStr">
         <is>
           <t>Dal &amp; Pulses</t>
         </is>
       </c>
-      <c r="D156" s="11" t="n">
+      <c r="D156" s="6" t="n">
         <v>103.04</v>
       </c>
-      <c r="E156" s="12" t="n">
+      <c r="E156" s="7" t="n">
         <v>16.23</v>
       </c>
-      <c r="F156" s="12" t="n">
-        <v>13.23</v>
-      </c>
-      <c r="G156" s="11" t="n">
-        <v>106.7271</v>
-      </c>
-      <c r="H156" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I156" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J156" s="13" t="inlineStr">
-        <is>
-          <t>discount 16% reliably below break-even — even the optimistic CI of its effect (marg β +0.0030 vs pay-threshold 0.0119) doesn't pay; trim to 2% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K156" s="11" t="n">
-        <v>73.99190856313503</v>
+      <c r="F156" s="7" t="n">
+        <v>16.23</v>
+      </c>
+      <c r="G156" s="6" t="n">
+        <v>103.0371</v>
+      </c>
+      <c r="H156" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I156" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J156" s="8" t="inlineStr">
+        <is>
+          <t>competitive defense - hold, do not cut</t>
+        </is>
+      </c>
+      <c r="K156" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="157">
@@ -23084,50 +23084,50 @@
       </c>
     </row>
     <row r="482">
-      <c r="A482" s="9" t="inlineStr">
+      <c r="A482" s="4" t="inlineStr">
         <is>
           <t>White Poha</t>
         </is>
       </c>
-      <c r="B482" s="10" t="inlineStr">
+      <c r="B482" s="5" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="C482" s="9" t="inlineStr">
+      <c r="C482" s="4" t="inlineStr">
         <is>
           <t>Poha</t>
         </is>
       </c>
-      <c r="D482" s="11" t="n">
+      <c r="D482" s="6" t="n">
         <v>80.83</v>
       </c>
-      <c r="E482" s="12" t="n">
+      <c r="E482" s="7" t="n">
         <v>10.19</v>
       </c>
-      <c r="F482" s="12" t="n">
-        <v>7.19</v>
-      </c>
-      <c r="G482" s="11" t="n">
-        <v>83.529</v>
-      </c>
-      <c r="H482" s="9" t="inlineStr">
-        <is>
-          <t>CUT</t>
-        </is>
-      </c>
-      <c r="I482" s="9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J482" s="13" t="inlineStr">
-        <is>
-          <t>discount 10% reliably below break-even — even the optimistic CI of its effect (marg β -0.0014 vs pay-threshold 0.0111) doesn't pay; trim to 0% (observed floor), volume held → net-rev gain</t>
-        </is>
-      </c>
-      <c r="K482" s="11" t="n">
-        <v>539.941060903733</v>
+      <c r="F482" s="7" t="n">
+        <v>10.19</v>
+      </c>
+      <c r="G482" s="6" t="n">
+        <v>80.82900000000001</v>
+      </c>
+      <c r="H482" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I482" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J482" s="8" t="inlineStr">
+        <is>
+          <t>competitive defense - hold, do not cut</t>
+        </is>
+      </c>
+      <c r="K482" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="483">
@@ -28166,7 +28166,7 @@
         </is>
       </c>
       <c r="K590" s="15" t="n">
-        <v>32910.16970608517</v>
+        <v>32163.78379096613</v>
       </c>
     </row>
   </sheetData>
@@ -28224,7 +28224,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>1213421.6965</v>
+        <v>1214296.0105</v>
       </c>
     </row>
     <row r="6">
@@ -28234,7 +28234,7 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>13.55027489235016</v>
+        <v>13.5600383530468</v>
       </c>
     </row>
     <row r="7">
@@ -28254,7 +28254,7 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>41168.19949999987</v>
+        <v>40293.88549999986</v>
       </c>
     </row>
     <row r="9"/>

</xml_diff>

<commit_message>
config: 12% weekly discount-spend cap + documented hero-SKU slot
Bake the chosen first-wave budget ceiling (DEFAULT_BUDGET_PCT_CAP=0.12) into
v4_config so it's not a flag to remember; tracker precedence is now
--budget_pct > config default > live baseline. At 12% (below current ~14%)
day one reads RED = 'over your new ceiling, glide down' (blocks reinvests only,
0 this week; cuts intact at 48 / ₹32k/wk). STRATEGIC_SKUS documented as the
hero-SKU shield, still [] pending the owner's flagship IDs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
+++ b/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
@@ -100,7 +100,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DD8B1A"/>
+        <fgColor rgb="00D64545"/>
       </patternFill>
     </fill>
   </fills>
@@ -28244,7 +28244,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>14.01</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -28254,7 +28254,7 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>40293.88549999986</v>
+        <v>-139700.8105000001</v>
       </c>
     </row>
     <row r="9"/>
@@ -28266,7 +28266,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>AMBER</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="C10" s="21" t="n"/>

</xml_diff>

<commit_message>
feat(loop): advance weekly loop to W3 — frozen baselines, round-2 scenarios, 12% budget cap
One full turn of the operating loop on run 20260711_221318 (model outputs
numerically identical to 20260705_161703 — reproducibility receipt):

- tracker_history.csv: W1→W3, schema widened 11→18 cols (baseline/actual
  OSA-SOV, strikes, cell_status)
- baselines.json (new): pre-action baselines frozen once for all 585 cells —
  the Gap-1 mean-reversion defense
- pricing/scenarios/round_02/ (new) + 9 rows in negotiation_log.csv; reco
  CSVs identical to round_01 (no negotiation feedback ingested yet)
- BUDGET_PLAN.md: discount spend cap 10% → 12% of revenue (aligns with
  DEFAULT_BUDGET_PCT_CAP=0.12)
- challenger/validation/promo artifacts: run-stamp + solver-timing telemetry
  refresh only

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
+++ b/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
@@ -595,7 +595,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Weekly Discount Plan — W1</t>
+          <t>Weekly Discount Plan — W3</t>
         </is>
       </c>
     </row>
@@ -28644,7 +28644,7 @@
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
-          <t>This week (W1)</t>
+          <t>This week (W3)</t>
         </is>
       </c>
     </row>
@@ -28692,7 +28692,7 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>No festival window contains 2026-07-06 (W1); all 585 cells scored normally, budget uplift 0.0.</t>
+          <t>No festival window contains 2026-07-06 (W3); all 585 cells scored normally, budget uplift 0.0.</t>
         </is>
       </c>
     </row>
@@ -28908,7 +28908,7 @@
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Every Monday, run the weekly export from the tool. It produces this workbook, named with the week (e.g. this one is W1).</t>
+          <t>Every Monday, run the weekly export from the tool. It produces this workbook, named with the week (e.g. this one is W3).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(loop): reset tracker to the intentional W1 baseline
The W2 block was a side-effect of the settings fail-loud verification runs
(weekly_tracker.py auto-appends the next week). Reverted the four tracker
artifacts to their state at 274d762 so the real operating timeline starts
clean: 537 rows, W1 only, 24 cuts / 513 holds, 0 scored; baselines.json
stays absent (re-freezes on the first --actuals run). The next genuine Monday
cycle is W2, not W3.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
+++ b/DISCOUNT_PLAN/WEEKLY_TRACKER.xlsx
@@ -595,7 +595,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Weekly Discount Plan — W2</t>
+          <t>Weekly Discount Plan — W1</t>
         </is>
       </c>
     </row>
@@ -26388,7 +26388,7 @@
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
-          <t>This week (W2)</t>
+          <t>This week (W1)</t>
         </is>
       </c>
     </row>
@@ -26436,7 +26436,7 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>No festival window contains 2026-07-13 (W2); all 537 cells scored normally, budget uplift 0.0.</t>
+          <t>No festival window contains 2026-07-20 (W1); all 537 cells scored normally, budget uplift 0.0.</t>
         </is>
       </c>
     </row>
@@ -26652,7 +26652,7 @@
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Every Monday, run the weekly export from the tool. It produces this workbook, named with the week (e.g. this one is W2).</t>
+          <t>Every Monday, run the weekly export from the tool. It produces this workbook, named with the week (e.g. this one is W1).</t>
         </is>
       </c>
     </row>

</xml_diff>